<commit_message>
resolução de bugs e aprimoramento de UX
</commit_message>
<xml_diff>
--- a/log_cancelamentos.xlsx
+++ b/log_cancelamentos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,6 +515,33 @@
         </is>
       </c>
       <c r="E4" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>03/06/2026 13:49</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>LUCAS NOBREGA ALBUQUERQUE</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>(55) 83996-4354</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Problemas técnicos na plataforma ou instabilidade de internet</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>PENDENTE</t>
         </is>

</xml_diff>